<commit_message>
App web: login por convite e tela de cargas; migrations 0002 e 0003
- 0002: controle de migrations, token de acesso e sessão, staging das cargas
- 0003: aplicar_carga (valida e aplica a planilha, tudo ou nada) e criar_rodada
- 0001: search_path nas funções; meta de consultor total com chave própria
- web/: Next.js 16, login por link de uso único com confirmação, /admin/cargas, /admin/usuarios
- scripts: npm run migrar, npm run link -- email
- testes em PGlite (12) e modelo de carga sem notas nas abas de dados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLw9XY3Ph6PE4HvNMuHGzq
</commit_message>
<xml_diff>
--- a/cargas/modelos_cargas.xlsx
+++ b/cargas/modelos_cargas.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,10 +56,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00667085"/>
     </font>
   </fonts>
   <fills count="3">
@@ -101,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,7 +107,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -478,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -687,6 +682,76 @@
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>O que vai em cada aba</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>hierarquia: Uma linha por dealer. Um grupo por marca (grupo com Fiat e CJDR = dois códigos de grupo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>consultores: perfil: cpv, cna, cne, fi. E-mail preenchido cria o usuário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>carteira: Por rodada. CNA/CNE com carteira herdada: repetir as linhas do CPV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>usuarios: grupos: códigos separados por ; (perfil grupo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>base21: Por rodada, dealer × PN. Valores de item (categoria, qme, preço, condição) iguais em todas as linhas do mesmo PN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>catalogo_fornecedor: Por rodada. Sem colunas de demanda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>metas: Por rodada, grupo × categoria, em R$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>metas_consultor: Opcional, para os rankings. categoria vazia = total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>csps: Pós-evento: extração do CSPS. Colunas extras são ignoradas.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -698,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -757,13 +822,6 @@
       <c r="E2" s="4" t="inlineStr">
         <is>
           <t>2026-12-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Pós-evento: extração do CSPS. Colunas extras são ignoradas.</t>
         </is>
       </c>
     </row>
@@ -779,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1044,13 +1102,6 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Uma linha por dealer. Um grupo por marca (grupo com Fiat e CJDR = dois códigos de grupo).</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:L4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1063,7 +1114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1158,13 +1209,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>perfil: cpv, cna, cne, fi. E-mail preenchido cria o usuário.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:F3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1177,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1229,13 +1273,6 @@
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>G0001</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Por rodada. CNA/CNE com carteira herdada: repetir as linhas do CPV.</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1396,13 +1433,6 @@
       </c>
       <c r="G5" s="6" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>grupos: códigos separados por ; (perfil grupo).</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1415,7 +1445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1535,7 +1565,7 @@
       <c r="F2" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="7" t="n">
         <v>18.9</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -1587,7 +1617,7 @@
       <c r="F3" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="7" t="n">
         <v>32.5</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -1641,7 +1671,7 @@
       <c r="F4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="7" t="n">
         <v>18.9</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -1663,13 +1693,6 @@
         <v>0</v>
       </c>
       <c r="N4" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Por rodada, dealer × PN. Valores de item (categoria, qme, preço, condição) iguais em todas as linhas do mesmo PN.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N4"/>
@@ -1683,7 +1706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1779,7 +1802,7 @@
       <c r="F2" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="7" t="n">
         <v>24.9</v>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -1790,13 +1813,6 @@
       <c r="I2" s="4" t="inlineStr"/>
       <c r="J2" s="4" t="n">
         <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Por rodada. Sem colunas de demanda.</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1811,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1847,7 +1863,7 @@
           <t>PECAS</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="7" t="n">
         <v>250000</v>
       </c>
     </row>
@@ -1862,7 +1878,7 @@
           <t>ACESSORIOS</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="7" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -1877,15 +1893,8 @@
           <t>PECAS</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="7" t="n">
         <v>180000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Por rodada, grupo × categoria, em R$.</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -1900,7 +1909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1932,7 +1941,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr"/>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="7" t="n">
         <v>1500000</v>
       </c>
     </row>
@@ -1947,15 +1956,8 @@
           <t>ACESSORIOS</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="7" t="n">
         <v>120000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Opcional, para os rankings. categoria vazia = total.</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>